<commit_message>
update of 13th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F173810-A75F-420A-9609-C7EA78174514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D1B51D-79DE-480B-AA8C-114FD7438A86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="87">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -293,6 +293,9 @@
   </si>
   <si>
     <t>team meeting done</t>
+  </si>
+  <si>
+    <t>injured</t>
   </si>
 </sst>
 </file>
@@ -2276,26 +2279,50 @@
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
+      <c r="A32" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B32" s="14">
+        <v>480</v>
+      </c>
+      <c r="C32" s="14">
+        <v>150</v>
+      </c>
+      <c r="D32" s="14">
+        <v>180</v>
+      </c>
+      <c r="E32" s="14">
+        <v>100</v>
+      </c>
+      <c r="F32" s="14">
+        <v>0</v>
+      </c>
+      <c r="G32" s="14">
+        <v>0</v>
+      </c>
+      <c r="H32" s="14">
+        <v>300</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
+        <v>1210</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="17"/>
+        <v>230</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>

</xml_diff>

<commit_message>
update of 14th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D1B51D-79DE-480B-AA8C-114FD7438A86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A2D58A-F205-45ED-8207-D255277B2233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="88">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -296,6 +296,9 @@
   </si>
   <si>
     <t>injured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mars </t>
   </si>
 </sst>
 </file>
@@ -2325,26 +2328,50 @@
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="15" t="str">
+      <c r="A33" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B33" s="14">
+        <v>480</v>
+      </c>
+      <c r="C33" s="14">
+        <v>150</v>
+      </c>
+      <c r="D33" s="14">
+        <v>210</v>
+      </c>
+      <c r="E33" s="14">
+        <v>100</v>
+      </c>
+      <c r="F33" s="14">
+        <v>200</v>
+      </c>
+      <c r="G33" s="14">
+        <v>4</v>
+      </c>
+      <c r="H33" s="14">
+        <v>300</v>
+      </c>
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N33" s="17" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>

</xml_diff>

<commit_message>
update of 15th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A2D58A-F205-45ED-8207-D255277B2233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69EE59E-E23D-43D3-8290-4556704DB7D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -299,6 +299,9 @@
   </si>
   <si>
     <t xml:space="preserve">mars </t>
+  </si>
+  <si>
+    <t xml:space="preserve">game mode </t>
   </si>
 </sst>
 </file>
@@ -2374,26 +2377,50 @@
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+      <c r="A34" s="13">
+        <v>46280</v>
+      </c>
+      <c r="B34" s="14">
+        <v>480</v>
+      </c>
+      <c r="C34" s="14">
+        <v>90</v>
+      </c>
+      <c r="D34" s="14">
+        <v>120</v>
+      </c>
+      <c r="E34" s="14">
+        <v>200</v>
+      </c>
+      <c r="F34" s="14">
+        <v>350</v>
+      </c>
+      <c r="G34" s="14">
+        <v>7</v>
+      </c>
+      <c r="H34" s="14">
+        <v>200</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="13"/>

</xml_diff>

<commit_message>
update of 16th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69EE59E-E23D-43D3-8290-4556704DB7D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44388BBF-5105-4023-8A4F-177B63837848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t xml:space="preserve">game mode </t>
+  </si>
+  <si>
+    <t>lets begin my data my story</t>
   </si>
 </sst>
 </file>
@@ -2423,26 +2426,50 @@
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+      <c r="A35" s="13">
+        <v>46281</v>
+      </c>
+      <c r="B35" s="14">
+        <v>480</v>
+      </c>
+      <c r="C35" s="14">
+        <v>30</v>
+      </c>
+      <c r="D35" s="14">
+        <v>180</v>
+      </c>
+      <c r="E35" s="14">
+        <v>150</v>
+      </c>
+      <c r="F35" s="14">
+        <v>350</v>
+      </c>
+      <c r="G35" s="14">
+        <v>7</v>
+      </c>
+      <c r="H35" s="14">
+        <v>250</v>
+      </c>
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N35" s="17" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="13"/>

</xml_diff>

<commit_message>
update of 17th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44388BBF-5105-4023-8A4F-177B63837848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497896B9-A934-4C82-BB70-39E3052E213C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="91">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -305,6 +305,9 @@
   </si>
   <si>
     <t>lets begin my data my story</t>
+  </si>
+  <si>
+    <t>memories</t>
   </si>
 </sst>
 </file>
@@ -2472,26 +2475,50 @@
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+      <c r="A36" s="13">
+        <v>46282</v>
+      </c>
+      <c r="B36" s="14">
+        <v>480</v>
+      </c>
+      <c r="C36" s="14">
+        <v>30</v>
+      </c>
+      <c r="D36" s="14">
+        <v>240</v>
+      </c>
+      <c r="E36" s="14">
+        <v>100</v>
+      </c>
+      <c r="F36" s="14">
+        <v>200</v>
+      </c>
+      <c r="G36" s="14">
+        <v>4</v>
+      </c>
+      <c r="H36" s="14">
+        <v>390</v>
+      </c>
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N36" s="17" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="13"/>

</xml_diff>

<commit_message>
update of 18th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497896B9-A934-4C82-BB70-39E3052E213C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF389CD4-C550-4262-B797-73295BDE24DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="92">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -308,6 +308,9 @@
   </si>
   <si>
     <t>memories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As Usual CA </t>
   </si>
 </sst>
 </file>
@@ -2521,26 +2524,50 @@
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+      <c r="A37" s="13">
+        <v>46283</v>
+      </c>
+      <c r="B37" s="14">
+        <v>480</v>
+      </c>
+      <c r="C37" s="14">
+        <v>60</v>
+      </c>
+      <c r="D37" s="14">
+        <v>240</v>
+      </c>
+      <c r="E37" s="14">
+        <v>100</v>
+      </c>
+      <c r="F37" s="14">
+        <v>250</v>
+      </c>
+      <c r="G37" s="14">
+        <v>5</v>
+      </c>
+      <c r="H37" s="14">
+        <v>310</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N37" s="17" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="13"/>

</xml_diff>

<commit_message>
update of 19th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF389CD4-C550-4262-B797-73295BDE24DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65AF6785-F3C3-41A0-A3C1-8F693C2DF300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="93">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t xml:space="preserve">As Usual CA </t>
+  </si>
+  <si>
+    <t>Growing</t>
   </si>
 </sst>
 </file>
@@ -2570,26 +2573,50 @@
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+      <c r="A38" s="13">
+        <v>46284</v>
+      </c>
+      <c r="B38" s="14">
+        <v>480</v>
+      </c>
+      <c r="C38" s="14">
+        <v>60</v>
+      </c>
+      <c r="D38" s="14">
+        <v>240</v>
+      </c>
+      <c r="E38" s="14">
+        <v>100</v>
+      </c>
+      <c r="F38" s="14">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14">
+        <v>0</v>
+      </c>
+      <c r="H38" s="14">
+        <v>300</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>1180</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="17"/>
+        <v>260</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N38" s="17" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="13"/>

</xml_diff>

<commit_message>
update of 20th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65AF6785-F3C3-41A0-A3C1-8F693C2DF300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEAC09DB-0738-4D8D-B805-6CB91C7D2EB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="94">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t>Growing</t>
+  </si>
+  <si>
+    <t>working on data project</t>
   </si>
 </sst>
 </file>
@@ -2619,26 +2622,50 @@
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+      <c r="A39" s="13">
+        <v>46285</v>
+      </c>
+      <c r="B39" s="14">
+        <v>480</v>
+      </c>
+      <c r="C39" s="14">
+        <v>150</v>
+      </c>
+      <c r="D39" s="14">
+        <v>250</v>
+      </c>
+      <c r="E39" s="14">
+        <v>150</v>
+      </c>
+      <c r="F39" s="14">
+        <v>0</v>
+      </c>
+      <c r="G39" s="14">
+        <v>0</v>
+      </c>
+      <c r="H39" s="14">
+        <v>250</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>1280</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="17"/>
+        <v>160</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N39" s="17" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" s="13"/>

</xml_diff>

<commit_message>
update of 21st Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEAC09DB-0738-4D8D-B805-6CB91C7D2EB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197360B6-E4D5-47BD-A9E7-8212A1135071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="95">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -317,6 +317,9 @@
   </si>
   <si>
     <t>working on data project</t>
+  </si>
+  <si>
+    <t>going with the flow</t>
   </si>
 </sst>
 </file>
@@ -2668,26 +2671,50 @@
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+      <c r="A40" s="13">
+        <v>46286</v>
+      </c>
+      <c r="B40" s="14">
+        <v>480</v>
+      </c>
+      <c r="C40" s="14">
+        <v>60</v>
+      </c>
+      <c r="D40" s="14">
+        <v>250</v>
+      </c>
+      <c r="E40" s="14">
+        <v>150</v>
+      </c>
+      <c r="F40" s="14">
+        <v>200</v>
+      </c>
+      <c r="G40" s="14">
+        <v>4</v>
+      </c>
+      <c r="H40" s="14">
+        <v>300</v>
+      </c>
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N40" s="17" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="13"/>

</xml_diff>

<commit_message>
update of 23th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197360B6-E4D5-47BD-A9E7-8212A1135071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3500093B-33FE-4317-8B6E-9631C9E5FCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="95">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2717,48 +2717,96 @@
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="13"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+      <c r="A41" s="13">
+        <v>46287</v>
+      </c>
+      <c r="B41" s="14">
+        <v>480</v>
+      </c>
+      <c r="C41" s="14">
+        <v>60</v>
+      </c>
+      <c r="D41" s="14">
+        <v>120</v>
+      </c>
+      <c r="E41" s="14">
+        <v>200</v>
+      </c>
+      <c r="F41" s="14">
+        <v>350</v>
+      </c>
+      <c r="G41" s="14">
+        <v>7</v>
+      </c>
+      <c r="H41" s="14">
+        <v>230</v>
+      </c>
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N41" s="17" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="13"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="15" t="str">
+      <c r="A42" s="13">
+        <v>46288</v>
+      </c>
+      <c r="B42" s="14">
+        <v>480</v>
+      </c>
+      <c r="C42" s="14">
+        <v>60</v>
+      </c>
+      <c r="D42" s="14">
+        <v>120</v>
+      </c>
+      <c r="E42" s="14">
+        <v>200</v>
+      </c>
+      <c r="F42" s="14">
+        <v>350</v>
+      </c>
+      <c r="G42" s="14">
+        <v>7</v>
+      </c>
+      <c r="H42" s="14">
+        <v>230</v>
+      </c>
+      <c r="I42" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J42" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K42" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L42" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N42" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="13"/>

</xml_diff>

<commit_message>
update of 25th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3500093B-33FE-4317-8B6E-9631C9E5FCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62329C0-02BC-48D3-8D06-75CD6FFA06AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="97">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -320,6 +320,12 @@
   </si>
   <si>
     <t>going with the flow</t>
+  </si>
+  <si>
+    <t>As Usual CA  Prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minor project </t>
   </si>
 </sst>
 </file>
@@ -2809,48 +2815,96 @@
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="13"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="15" t="str">
+      <c r="A43" s="13">
+        <v>46289</v>
+      </c>
+      <c r="B43" s="14">
+        <v>480</v>
+      </c>
+      <c r="C43" s="14">
+        <v>150</v>
+      </c>
+      <c r="D43" s="14">
+        <v>240</v>
+      </c>
+      <c r="E43" s="14">
+        <v>100</v>
+      </c>
+      <c r="F43" s="14">
+        <v>200</v>
+      </c>
+      <c r="G43" s="14">
+        <v>4</v>
+      </c>
+      <c r="H43" s="14">
+        <v>270</v>
+      </c>
+      <c r="I43" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J43" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
-      <c r="N43" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L43" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M43" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N43" s="17" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="13"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="15" t="str">
+      <c r="A44" s="13">
+        <v>46290</v>
+      </c>
+      <c r="B44" s="14">
+        <v>480</v>
+      </c>
+      <c r="C44" s="14">
+        <v>60</v>
+      </c>
+      <c r="D44" s="14">
+        <v>200</v>
+      </c>
+      <c r="E44" s="14">
+        <v>300</v>
+      </c>
+      <c r="F44" s="14">
+        <v>250</v>
+      </c>
+      <c r="G44" s="14">
+        <v>5</v>
+      </c>
+      <c r="H44" s="14">
+        <v>150</v>
+      </c>
+      <c r="I44" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J44" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
-      <c r="M44" s="16"/>
-      <c r="N44" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K44" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L44" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M44" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N44" s="17" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="13"/>

</xml_diff>

<commit_message>
update of 27th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62329C0-02BC-48D3-8D06-75CD6FFA06AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D00C6C5A-7E64-4330-9002-E54025D89533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="98">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -326,6 +326,9 @@
   </si>
   <si>
     <t xml:space="preserve">Minor project </t>
+  </si>
+  <si>
+    <t>going home</t>
   </si>
 </sst>
 </file>
@@ -2907,48 +2910,96 @@
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="13"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="15" t="str">
+      <c r="A45" s="13">
+        <v>46291</v>
+      </c>
+      <c r="B45" s="14">
+        <v>480</v>
+      </c>
+      <c r="C45" s="14">
+        <v>150</v>
+      </c>
+      <c r="D45" s="14">
+        <v>200</v>
+      </c>
+      <c r="E45" s="14">
+        <v>300</v>
+      </c>
+      <c r="F45" s="14">
+        <v>0</v>
+      </c>
+      <c r="G45" s="14">
+        <v>0</v>
+      </c>
+      <c r="H45" s="14">
+        <v>300</v>
+      </c>
+      <c r="I45" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="15" t="str">
+        <v>1430</v>
+      </c>
+      <c r="J45" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="17"/>
+        <v>10</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L45" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M45" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N45" s="17" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="13"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="15" t="str">
+      <c r="A46" s="13">
+        <v>46292</v>
+      </c>
+      <c r="B46" s="14">
+        <v>480</v>
+      </c>
+      <c r="C46" s="14">
+        <v>150</v>
+      </c>
+      <c r="D46" s="14">
+        <v>180</v>
+      </c>
+      <c r="E46" s="14">
+        <v>280</v>
+      </c>
+      <c r="F46" s="14">
+        <v>0</v>
+      </c>
+      <c r="G46" s="14">
+        <v>0</v>
+      </c>
+      <c r="H46" s="14">
+        <v>300</v>
+      </c>
+      <c r="I46" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="15" t="str">
+        <v>1390</v>
+      </c>
+      <c r="J46" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="17"/>
+        <v>50</v>
+      </c>
+      <c r="K46" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L46" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M46" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N46" s="17" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="13"/>

</xml_diff>

<commit_message>
update till 30th Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D00C6C5A-7E64-4330-9002-E54025D89533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC1593F-CC27-4D93-8F7B-161407EA6198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="101">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -329,6 +329,15 @@
   </si>
   <si>
     <t>going home</t>
+  </si>
+  <si>
+    <t>sometihng happening in college</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unfortunate situation </t>
+  </si>
+  <si>
+    <t>back home</t>
   </si>
 </sst>
 </file>
@@ -3002,70 +3011,142 @@
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="13"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="15" t="str">
+      <c r="A47" s="13">
+        <v>46293</v>
+      </c>
+      <c r="B47" s="14">
+        <v>400</v>
+      </c>
+      <c r="C47" s="14">
+        <v>200</v>
+      </c>
+      <c r="D47" s="14">
+        <v>100</v>
+      </c>
+      <c r="E47" s="14">
+        <v>100</v>
+      </c>
+      <c r="F47" s="14">
+        <v>0</v>
+      </c>
+      <c r="G47" s="14">
+        <v>0</v>
+      </c>
+      <c r="H47" s="14">
+        <v>640</v>
+      </c>
+      <c r="I47" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J47" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K47" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L47" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M47" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N47" s="17" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="13"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="15" t="str">
+      <c r="A48" s="13">
+        <v>46294</v>
+      </c>
+      <c r="B48" s="14">
+        <v>400</v>
+      </c>
+      <c r="C48" s="14">
+        <v>200</v>
+      </c>
+      <c r="D48" s="14">
+        <v>100</v>
+      </c>
+      <c r="E48" s="14">
+        <v>100</v>
+      </c>
+      <c r="F48" s="14">
+        <v>0</v>
+      </c>
+      <c r="G48" s="14">
+        <v>0</v>
+      </c>
+      <c r="H48" s="14">
+        <v>640</v>
+      </c>
+      <c r="I48" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J48" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16"/>
-      <c r="M48" s="16"/>
-      <c r="N48" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K48" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L48" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M48" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N48" s="17" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="13"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15" t="str">
+      <c r="A49" s="13">
+        <v>46295</v>
+      </c>
+      <c r="B49" s="14">
+        <v>400</v>
+      </c>
+      <c r="C49" s="14">
+        <v>200</v>
+      </c>
+      <c r="D49" s="14">
+        <v>100</v>
+      </c>
+      <c r="E49" s="14">
+        <v>200</v>
+      </c>
+      <c r="F49" s="14">
+        <v>0</v>
+      </c>
+      <c r="G49" s="14">
+        <v>0</v>
+      </c>
+      <c r="H49" s="14">
+        <v>540</v>
+      </c>
+      <c r="I49" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J49" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M49" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N49" s="17" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="13"/>

</xml_diff>

<commit_message>
update of 1st Aug
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC1593F-CC27-4D93-8F7B-161407EA6198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7AFCED7-A9C4-480C-BA9B-B68AB3EFDD9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="102">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -265,9 +265,6 @@
     <t>hostel room got boom</t>
   </si>
   <si>
-    <t xml:space="preserve"> September</t>
-  </si>
-  <si>
     <t>R&amp;D for new project</t>
   </si>
   <si>
@@ -338,6 +335,12 @@
   </si>
   <si>
     <t>back home</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> October</t>
+  </si>
+  <si>
+    <t>enjyoing few moments</t>
   </si>
 </sst>
 </file>
@@ -1058,7 +1061,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="G3" s="20"/>
     </row>
@@ -1949,7 +1952,7 @@
         <v>58</v>
       </c>
       <c r="N23" s="17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
@@ -1995,7 +1998,7 @@
         <v>58</v>
       </c>
       <c r="N24" s="17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
@@ -2041,7 +2044,7 @@
         <v>56</v>
       </c>
       <c r="N25" s="17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
@@ -2087,7 +2090,7 @@
         <v>56</v>
       </c>
       <c r="N26" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
@@ -2133,7 +2136,7 @@
         <v>56</v>
       </c>
       <c r="N27" s="17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
@@ -2179,7 +2182,7 @@
         <v>58</v>
       </c>
       <c r="N28" s="17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
@@ -2225,7 +2228,7 @@
         <v>58</v>
       </c>
       <c r="N29" s="17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
@@ -2271,7 +2274,7 @@
         <v>58</v>
       </c>
       <c r="N30" s="17" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
@@ -2317,7 +2320,7 @@
         <v>58</v>
       </c>
       <c r="N31" s="17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
@@ -2363,7 +2366,7 @@
         <v>58</v>
       </c>
       <c r="N32" s="17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
@@ -2409,7 +2412,7 @@
         <v>58</v>
       </c>
       <c r="N33" s="17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
@@ -2455,7 +2458,7 @@
         <v>58</v>
       </c>
       <c r="N34" s="17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
@@ -2501,7 +2504,7 @@
         <v>56</v>
       </c>
       <c r="N35" s="17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
@@ -2547,7 +2550,7 @@
         <v>56</v>
       </c>
       <c r="N36" s="17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
@@ -2593,7 +2596,7 @@
         <v>58</v>
       </c>
       <c r="N37" s="17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
@@ -2639,7 +2642,7 @@
         <v>58</v>
       </c>
       <c r="N38" s="17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
@@ -2685,7 +2688,7 @@
         <v>56</v>
       </c>
       <c r="N39" s="17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
@@ -2731,7 +2734,7 @@
         <v>58</v>
       </c>
       <c r="N40" s="17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
@@ -2869,7 +2872,7 @@
         <v>56</v>
       </c>
       <c r="N43" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
@@ -2915,7 +2918,7 @@
         <v>56</v>
       </c>
       <c r="N44" s="17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
@@ -2961,7 +2964,7 @@
         <v>56</v>
       </c>
       <c r="N45" s="17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
@@ -3007,7 +3010,7 @@
         <v>58</v>
       </c>
       <c r="N46" s="17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
@@ -3053,7 +3056,7 @@
         <v>58</v>
       </c>
       <c r="N47" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
@@ -3099,7 +3102,7 @@
         <v>58</v>
       </c>
       <c r="N48" s="17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
@@ -3145,30 +3148,54 @@
         <v>58</v>
       </c>
       <c r="N49" s="17" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A50" s="13">
+        <v>46296</v>
+      </c>
+      <c r="B50" s="14">
+        <v>480</v>
+      </c>
+      <c r="C50" s="14">
+        <v>200</v>
+      </c>
+      <c r="D50" s="14">
+        <v>200</v>
+      </c>
+      <c r="E50" s="14">
         <v>100</v>
       </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="13"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="15" t="str">
+      <c r="F50" s="14">
+        <v>0</v>
+      </c>
+      <c r="G50" s="14">
+        <v>0</v>
+      </c>
+      <c r="H50" s="14">
+        <v>400</v>
+      </c>
+      <c r="I50" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="15" t="str">
+        <v>1380</v>
+      </c>
+      <c r="J50" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="17"/>
+        <v>60</v>
+      </c>
+      <c r="K50" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L50" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M50" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N50" s="17" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="13"/>

</xml_diff>

<commit_message>
update of 02th october
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7AFCED7-A9C4-480C-BA9B-B68AB3EFDD9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83BF307D-AAAD-49E7-B26F-0D13D3200E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="103">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -341,6 +341,9 @@
   </si>
   <si>
     <t>enjyoing few moments</t>
+  </si>
+  <si>
+    <t>working</t>
   </si>
 </sst>
 </file>
@@ -3198,26 +3201,50 @@
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="13"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="15" t="str">
+      <c r="A51" s="13">
+        <v>46297</v>
+      </c>
+      <c r="B51" s="14">
+        <v>480</v>
+      </c>
+      <c r="C51" s="14">
+        <v>150</v>
+      </c>
+      <c r="D51" s="14">
+        <v>100</v>
+      </c>
+      <c r="E51" s="14">
+        <v>200</v>
+      </c>
+      <c r="F51" s="14">
+        <v>0</v>
+      </c>
+      <c r="G51" s="14">
+        <v>0</v>
+      </c>
+      <c r="H51" s="14">
+        <v>400</v>
+      </c>
+      <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
+        <v>1330</v>
+      </c>
+      <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="17"/>
+        <v>110</v>
+      </c>
+      <c r="K51" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M51" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N51" s="17" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="13"/>

</xml_diff>

<commit_message>
update till 12th october
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83BF307D-AAAD-49E7-B26F-0D13D3200E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15644507-19B5-4E3E-8E2A-98796C694D32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="113">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -344,6 +344,36 @@
   </si>
   <si>
     <t>working</t>
+  </si>
+  <si>
+    <t>village moments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">happy me </t>
+  </si>
+  <si>
+    <t xml:space="preserve">return back to city </t>
+  </si>
+  <si>
+    <t>online classes ongoing</t>
+  </si>
+  <si>
+    <t>working mode</t>
+  </si>
+  <si>
+    <t>festival molde</t>
+  </si>
+  <si>
+    <t>nice all good</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inside the train </t>
+  </si>
+  <si>
+    <t>reached delhi</t>
+  </si>
+  <si>
+    <t>back to college</t>
   </si>
 </sst>
 </file>
@@ -3247,224 +3277,464 @@
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="13"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="15" t="str">
+      <c r="A52" s="13">
+        <v>46298</v>
+      </c>
+      <c r="B52" s="14">
+        <v>480</v>
+      </c>
+      <c r="C52" s="14">
+        <v>200</v>
+      </c>
+      <c r="D52" s="14">
+        <v>100</v>
+      </c>
+      <c r="E52" s="14">
+        <v>160</v>
+      </c>
+      <c r="F52" s="14">
+        <v>0</v>
+      </c>
+      <c r="G52" s="14">
+        <v>0</v>
+      </c>
+      <c r="H52" s="14">
+        <v>400</v>
+      </c>
+      <c r="I52" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
+        <v>1340</v>
+      </c>
+      <c r="J52" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="17"/>
+        <v>100</v>
+      </c>
+      <c r="K52" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M52" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N52" s="17" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="13"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="15" t="str">
+      <c r="A53" s="13">
+        <v>46299</v>
+      </c>
+      <c r="B53" s="14">
+        <v>480</v>
+      </c>
+      <c r="C53" s="14">
+        <v>500</v>
+      </c>
+      <c r="D53" s="14">
+        <v>100</v>
+      </c>
+      <c r="E53" s="14">
+        <v>150</v>
+      </c>
+      <c r="F53" s="14">
+        <v>0</v>
+      </c>
+      <c r="G53" s="14">
+        <v>0</v>
+      </c>
+      <c r="H53" s="14">
+        <v>210</v>
+      </c>
+      <c r="I53" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J53" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K53" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L53" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M53" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N53" s="17" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="13"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="14"/>
-      <c r="I54" s="15" t="str">
+      <c r="A54" s="13">
+        <v>46300</v>
+      </c>
+      <c r="B54" s="14">
+        <v>400</v>
+      </c>
+      <c r="C54" s="14">
+        <v>300</v>
+      </c>
+      <c r="D54" s="14">
+        <v>100</v>
+      </c>
+      <c r="E54" s="14">
+        <v>150</v>
+      </c>
+      <c r="F54" s="14">
+        <v>200</v>
+      </c>
+      <c r="G54" s="14">
+        <v>4</v>
+      </c>
+      <c r="H54" s="14">
+        <v>290</v>
+      </c>
+      <c r="I54" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J54" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="16"/>
-      <c r="L54" s="16"/>
-      <c r="M54" s="16"/>
-      <c r="N54" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K54" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L54" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M54" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N54" s="17" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="13"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="15" t="str">
+      <c r="A55" s="13">
+        <v>46301</v>
+      </c>
+      <c r="B55" s="14">
+        <v>400</v>
+      </c>
+      <c r="C55" s="14">
+        <v>60</v>
+      </c>
+      <c r="D55" s="14">
+        <v>200</v>
+      </c>
+      <c r="E55" s="14">
+        <v>220</v>
+      </c>
+      <c r="F55" s="14">
+        <v>350</v>
+      </c>
+      <c r="G55" s="14">
+        <v>7</v>
+      </c>
+      <c r="H55" s="14">
+        <v>210</v>
+      </c>
+      <c r="I55" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J55" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="16"/>
-      <c r="L55" s="16"/>
-      <c r="M55" s="16"/>
-      <c r="N55" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K55" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L55" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M55" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N55" s="17" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="13"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
-      <c r="F56" s="14"/>
-      <c r="G56" s="14"/>
-      <c r="H56" s="14"/>
-      <c r="I56" s="15" t="str">
+      <c r="A56" s="13">
+        <v>46302</v>
+      </c>
+      <c r="B56" s="14">
+        <v>400</v>
+      </c>
+      <c r="C56" s="14">
+        <v>60</v>
+      </c>
+      <c r="D56" s="14">
+        <v>130</v>
+      </c>
+      <c r="E56" s="14">
+        <v>200</v>
+      </c>
+      <c r="F56" s="14">
+        <v>350</v>
+      </c>
+      <c r="G56" s="14">
+        <v>7</v>
+      </c>
+      <c r="H56" s="14">
+        <v>300</v>
+      </c>
+      <c r="I56" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J56" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K56" s="16"/>
-      <c r="L56" s="16"/>
-      <c r="M56" s="16"/>
-      <c r="N56" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K56" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L56" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M56" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N56" s="17" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="13"/>
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="14"/>
-      <c r="H57" s="14"/>
-      <c r="I57" s="15" t="str">
+      <c r="A57" s="13">
+        <v>46303</v>
+      </c>
+      <c r="B57" s="14">
+        <v>400</v>
+      </c>
+      <c r="C57" s="14">
+        <v>200</v>
+      </c>
+      <c r="D57" s="14">
+        <v>130</v>
+      </c>
+      <c r="E57" s="14">
+        <v>200</v>
+      </c>
+      <c r="F57" s="14">
+        <v>200</v>
+      </c>
+      <c r="G57" s="14">
+        <v>4</v>
+      </c>
+      <c r="H57" s="14">
+        <v>310</v>
+      </c>
+      <c r="I57" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J57" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J57" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K57" s="16"/>
-      <c r="L57" s="16"/>
-      <c r="M57" s="16"/>
-      <c r="N57" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K57" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L57" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M57" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N57" s="17" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A58" s="13"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="15" t="str">
+      <c r="A58" s="13">
+        <v>46304</v>
+      </c>
+      <c r="B58" s="14">
+        <v>400</v>
+      </c>
+      <c r="C58" s="14">
+        <v>150</v>
+      </c>
+      <c r="D58" s="14">
+        <v>200</v>
+      </c>
+      <c r="E58" s="14">
+        <v>180</v>
+      </c>
+      <c r="F58" s="14">
+        <v>250</v>
+      </c>
+      <c r="G58" s="14">
+        <v>5</v>
+      </c>
+      <c r="H58" s="14">
+        <v>260</v>
+      </c>
+      <c r="I58" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J58" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J58" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K58" s="16"/>
-      <c r="L58" s="16"/>
-      <c r="M58" s="16"/>
-      <c r="N58" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K58" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L58" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M58" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N58" s="17" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A59" s="13"/>
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="14"/>
-      <c r="H59" s="14"/>
-      <c r="I59" s="15" t="str">
+      <c r="A59" s="13">
+        <v>46305</v>
+      </c>
+      <c r="B59" s="14">
+        <v>400</v>
+      </c>
+      <c r="C59" s="14">
+        <v>150</v>
+      </c>
+      <c r="D59" s="14">
+        <v>100</v>
+      </c>
+      <c r="E59" s="14">
+        <v>150</v>
+      </c>
+      <c r="F59" s="14">
+        <v>0</v>
+      </c>
+      <c r="G59" s="14">
+        <v>0</v>
+      </c>
+      <c r="H59" s="14">
+        <v>300</v>
+      </c>
+      <c r="I59" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J59" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J59" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K59" s="16"/>
-      <c r="L59" s="16"/>
-      <c r="M59" s="16"/>
-      <c r="N59" s="17"/>
+        <v>340</v>
+      </c>
+      <c r="K59" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L59" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M59" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N59" s="17" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A60" s="13"/>
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="14"/>
-      <c r="F60" s="14"/>
-      <c r="G60" s="14"/>
-      <c r="H60" s="14"/>
-      <c r="I60" s="15" t="str">
+      <c r="A60" s="13">
+        <v>46306</v>
+      </c>
+      <c r="B60" s="14">
+        <v>400</v>
+      </c>
+      <c r="C60" s="14">
+        <v>150</v>
+      </c>
+      <c r="D60" s="14">
+        <v>100</v>
+      </c>
+      <c r="E60" s="14">
+        <v>150</v>
+      </c>
+      <c r="F60" s="14">
+        <v>0</v>
+      </c>
+      <c r="G60" s="14">
+        <v>0</v>
+      </c>
+      <c r="H60" s="14">
+        <v>300</v>
+      </c>
+      <c r="I60" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J60" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J60" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K60" s="16"/>
-      <c r="L60" s="16"/>
-      <c r="M60" s="16"/>
-      <c r="N60" s="17"/>
+        <v>340</v>
+      </c>
+      <c r="K60" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L60" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M60" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N60" s="17" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="13"/>
-      <c r="B61" s="14"/>
-      <c r="C61" s="14"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
-      <c r="H61" s="14"/>
-      <c r="I61" s="15" t="str">
+      <c r="A61" s="13">
+        <v>46307</v>
+      </c>
+      <c r="B61" s="14">
+        <v>400</v>
+      </c>
+      <c r="C61" s="14">
+        <v>180</v>
+      </c>
+      <c r="D61" s="14">
+        <v>100</v>
+      </c>
+      <c r="E61" s="14">
+        <v>150</v>
+      </c>
+      <c r="F61" s="14">
+        <v>0</v>
+      </c>
+      <c r="G61" s="14">
+        <v>0</v>
+      </c>
+      <c r="H61" s="14">
+        <v>300</v>
+      </c>
+      <c r="I61" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J61" s="15" t="str">
+        <v>1130</v>
+      </c>
+      <c r="J61" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K61" s="16"/>
-      <c r="L61" s="16"/>
-      <c r="M61" s="16"/>
-      <c r="N61" s="17"/>
+        <v>310</v>
+      </c>
+      <c r="K61" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L61" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M61" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N61" s="17" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" s="13"/>

</xml_diff>

<commit_message>
update of 14th october
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15644507-19B5-4E3E-8E2A-98796C694D32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D606254-E03C-454D-9EF0-48A69EF977B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="114">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -374,6 +374,9 @@
   </si>
   <si>
     <t>back to college</t>
+  </si>
+  <si>
+    <t>mid  term going on</t>
   </si>
 </sst>
 </file>
@@ -3737,48 +3740,96 @@
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="13"/>
-      <c r="B62" s="14"/>
-      <c r="C62" s="14"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="14"/>
-      <c r="F62" s="14"/>
-      <c r="G62" s="14"/>
-      <c r="H62" s="14"/>
-      <c r="I62" s="15" t="str">
+      <c r="A62" s="13">
+        <v>46308</v>
+      </c>
+      <c r="B62" s="14">
+        <v>350</v>
+      </c>
+      <c r="C62" s="14">
+        <v>60</v>
+      </c>
+      <c r="D62" s="14">
+        <v>450</v>
+      </c>
+      <c r="E62" s="14">
+        <v>30</v>
+      </c>
+      <c r="F62" s="14">
+        <v>0</v>
+      </c>
+      <c r="G62" s="14">
+        <v>0</v>
+      </c>
+      <c r="H62" s="14">
+        <v>550</v>
+      </c>
+      <c r="I62" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J62" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J62" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K62" s="16"/>
-      <c r="L62" s="16"/>
-      <c r="M62" s="16"/>
-      <c r="N62" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K62" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L62" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M62" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N62" s="17" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="13"/>
-      <c r="B63" s="14"/>
-      <c r="C63" s="14"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="14"/>
-      <c r="F63" s="14"/>
-      <c r="G63" s="14"/>
-      <c r="H63" s="14"/>
-      <c r="I63" s="15" t="str">
+      <c r="A63" s="13">
+        <v>46309</v>
+      </c>
+      <c r="B63" s="14">
+        <v>350</v>
+      </c>
+      <c r="C63" s="14">
+        <v>60</v>
+      </c>
+      <c r="D63" s="14">
+        <v>450</v>
+      </c>
+      <c r="E63" s="14">
+        <v>30</v>
+      </c>
+      <c r="F63" s="14">
+        <v>0</v>
+      </c>
+      <c r="G63" s="14">
+        <v>0</v>
+      </c>
+      <c r="H63" s="14">
+        <v>550</v>
+      </c>
+      <c r="I63" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J63" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J63" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K63" s="16"/>
-      <c r="L63" s="16"/>
-      <c r="M63" s="16"/>
-      <c r="N63" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K63" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L63" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M63" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N63" s="17" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="13"/>

</xml_diff>

<commit_message>
update till 20th october
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D606254-E03C-454D-9EF0-48A69EF977B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A59864-8490-4659-8E24-4885806AF876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="118">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -377,6 +377,18 @@
   </si>
   <si>
     <t>mid  term going on</t>
+  </si>
+  <si>
+    <t>fun day</t>
+  </si>
+  <si>
+    <t>snooze</t>
+  </si>
+  <si>
+    <t>classes started after a month</t>
+  </si>
+  <si>
+    <t>good day</t>
   </si>
 </sst>
 </file>
@@ -3832,139 +3844,285 @@
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A64" s="13"/>
-      <c r="B64" s="14"/>
-      <c r="C64" s="14"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
-      <c r="F64" s="14"/>
-      <c r="G64" s="14"/>
-      <c r="H64" s="14"/>
-      <c r="I64" s="15" t="str">
+      <c r="A64" s="13">
+        <v>46310</v>
+      </c>
+      <c r="B64" s="14">
+        <v>400</v>
+      </c>
+      <c r="C64" s="14">
+        <v>60</v>
+      </c>
+      <c r="D64" s="14">
+        <v>450</v>
+      </c>
+      <c r="E64" s="14">
+        <v>60</v>
+      </c>
+      <c r="F64" s="14">
+        <v>0</v>
+      </c>
+      <c r="G64" s="14">
+        <v>0</v>
+      </c>
+      <c r="H64" s="14">
+        <v>470</v>
+      </c>
+      <c r="I64" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J64" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J64" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K64" s="16"/>
-      <c r="L64" s="16"/>
-      <c r="M64" s="16"/>
-      <c r="N64" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K64" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L64" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M64" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N64" s="17" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A65" s="13"/>
-      <c r="B65" s="14"/>
-      <c r="C65" s="14"/>
-      <c r="D65" s="14"/>
-      <c r="E65" s="14"/>
-      <c r="F65" s="14"/>
-      <c r="G65" s="14"/>
-      <c r="H65" s="14"/>
-      <c r="I65" s="15" t="str">
+      <c r="A65" s="13">
+        <v>46311</v>
+      </c>
+      <c r="B65" s="14">
+        <v>400</v>
+      </c>
+      <c r="C65" s="14">
+        <v>60</v>
+      </c>
+      <c r="D65" s="14">
+        <v>450</v>
+      </c>
+      <c r="E65" s="14">
+        <v>60</v>
+      </c>
+      <c r="F65" s="14">
+        <v>0</v>
+      </c>
+      <c r="G65" s="14">
+        <v>0</v>
+      </c>
+      <c r="H65" s="14">
+        <v>470</v>
+      </c>
+      <c r="I65" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J65" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J65" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K65" s="16"/>
-      <c r="L65" s="16"/>
-      <c r="M65" s="16"/>
-      <c r="N65" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K65" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L65" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M65" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N65" s="17" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A66" s="13"/>
-      <c r="B66" s="14"/>
-      <c r="C66" s="14"/>
-      <c r="D66" s="14"/>
-      <c r="E66" s="14"/>
-      <c r="F66" s="14"/>
-      <c r="G66" s="14"/>
-      <c r="H66" s="14"/>
-      <c r="I66" s="15" t="str">
+      <c r="A66" s="13">
+        <v>46312</v>
+      </c>
+      <c r="B66" s="14">
+        <v>400</v>
+      </c>
+      <c r="C66" s="14">
+        <v>60</v>
+      </c>
+      <c r="D66" s="14">
+        <v>450</v>
+      </c>
+      <c r="E66" s="14">
+        <v>60</v>
+      </c>
+      <c r="F66" s="14">
+        <v>0</v>
+      </c>
+      <c r="G66" s="14">
+        <v>0</v>
+      </c>
+      <c r="H66" s="14">
+        <v>470</v>
+      </c>
+      <c r="I66" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J66" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J66" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K66" s="16"/>
-      <c r="L66" s="16"/>
-      <c r="M66" s="16"/>
-      <c r="N66" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K66" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L66" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M66" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N66" s="17" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A67" s="13"/>
-      <c r="B67" s="14"/>
-      <c r="C67" s="14"/>
-      <c r="D67" s="14"/>
-      <c r="E67" s="14"/>
-      <c r="F67" s="14"/>
-      <c r="G67" s="14"/>
-      <c r="H67" s="14"/>
-      <c r="I67" s="15" t="str">
+      <c r="A67" s="13">
+        <v>46313</v>
+      </c>
+      <c r="B67" s="14">
+        <v>600</v>
+      </c>
+      <c r="C67" s="14">
+        <v>150</v>
+      </c>
+      <c r="D67" s="14">
+        <v>200</v>
+      </c>
+      <c r="E67" s="14">
+        <v>100</v>
+      </c>
+      <c r="F67" s="14">
+        <v>0</v>
+      </c>
+      <c r="G67" s="14">
+        <v>0</v>
+      </c>
+      <c r="H67" s="14">
+        <v>390</v>
+      </c>
+      <c r="I67" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J67" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J67" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K67" s="16"/>
-      <c r="L67" s="16"/>
-      <c r="M67" s="16"/>
-      <c r="N67" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K67" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L67" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M67" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N67" s="17" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A68" s="13"/>
-      <c r="B68" s="14"/>
-      <c r="C68" s="14"/>
-      <c r="D68" s="14"/>
-      <c r="E68" s="14"/>
-      <c r="F68" s="14"/>
-      <c r="G68" s="14"/>
-      <c r="H68" s="14"/>
-      <c r="I68" s="15" t="str">
+      <c r="A68" s="13">
+        <v>46314</v>
+      </c>
+      <c r="B68" s="14">
+        <v>480</v>
+      </c>
+      <c r="C68" s="14">
+        <v>150</v>
+      </c>
+      <c r="D68" s="14">
+        <v>200</v>
+      </c>
+      <c r="E68" s="14">
+        <v>100</v>
+      </c>
+      <c r="F68" s="14">
+        <v>150</v>
+      </c>
+      <c r="G68" s="14">
+        <v>3</v>
+      </c>
+      <c r="H68" s="14">
+        <v>360</v>
+      </c>
+      <c r="I68" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J68" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J68" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K68" s="16"/>
-      <c r="L68" s="16"/>
-      <c r="M68" s="16"/>
-      <c r="N68" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K68" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L68" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M68" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N68" s="17" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A69" s="13"/>
-      <c r="B69" s="14"/>
-      <c r="C69" s="14"/>
-      <c r="D69" s="14"/>
-      <c r="E69" s="14"/>
-      <c r="F69" s="14"/>
-      <c r="G69" s="14"/>
-      <c r="H69" s="14"/>
-      <c r="I69" s="15" t="str">
+      <c r="A69" s="13">
+        <v>46315</v>
+      </c>
+      <c r="B69" s="14">
+        <v>480</v>
+      </c>
+      <c r="C69" s="14">
+        <v>150</v>
+      </c>
+      <c r="D69" s="14">
+        <v>200</v>
+      </c>
+      <c r="E69" s="14">
+        <v>100</v>
+      </c>
+      <c r="F69" s="14">
+        <v>0</v>
+      </c>
+      <c r="G69" s="14">
+        <v>0</v>
+      </c>
+      <c r="H69" s="14">
+        <v>350</v>
+      </c>
+      <c r="I69" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J69" s="15" t="str">
+        <v>1280</v>
+      </c>
+      <c r="J69" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K69" s="16"/>
-      <c r="L69" s="16"/>
-      <c r="M69" s="16"/>
-      <c r="N69" s="17"/>
+        <v>160</v>
+      </c>
+      <c r="K69" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L69" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M69" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N69" s="17" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A70" s="13"/>
+      <c r="A70" s="13">
+        <v>46316</v>
+      </c>
       <c r="B70" s="14"/>
       <c r="C70" s="14"/>
       <c r="D70" s="14"/>

</xml_diff>

<commit_message>
update of 22th October
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A59864-8490-4659-8E24-4885806AF876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BAC59F4-56A7-4A86-BCF3-1C57AC27661C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="118">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4123,47 +4123,93 @@
       <c r="A70" s="13">
         <v>46316</v>
       </c>
-      <c r="B70" s="14"/>
-      <c r="C70" s="14"/>
-      <c r="D70" s="14"/>
-      <c r="E70" s="14"/>
-      <c r="F70" s="14"/>
-      <c r="G70" s="14"/>
-      <c r="H70" s="14"/>
-      <c r="I70" s="15" t="str">
+      <c r="B70" s="14">
+        <v>480</v>
+      </c>
+      <c r="C70" s="14">
+        <v>60</v>
+      </c>
+      <c r="D70" s="14">
+        <v>200</v>
+      </c>
+      <c r="E70" s="14">
+        <v>100</v>
+      </c>
+      <c r="F70" s="14">
+        <v>350</v>
+      </c>
+      <c r="G70" s="14">
+        <v>7</v>
+      </c>
+      <c r="H70" s="14">
+        <v>250</v>
+      </c>
+      <c r="I70" s="15">
         <f t="shared" ref="I70:I133" si="2">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
-        <v/>
-      </c>
-      <c r="J70" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J70" s="15">
         <f t="shared" ref="J70:J133" si="3">IF(I70="","",1440-I70)</f>
-        <v/>
-      </c>
-      <c r="K70" s="16"/>
-      <c r="L70" s="16"/>
-      <c r="M70" s="16"/>
-      <c r="N70" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K70" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L70" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M70" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N70" s="17" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A71" s="13"/>
-      <c r="B71" s="14"/>
-      <c r="C71" s="14"/>
-      <c r="D71" s="14"/>
-      <c r="E71" s="14"/>
-      <c r="F71" s="14"/>
-      <c r="G71" s="14"/>
-      <c r="H71" s="14"/>
-      <c r="I71" s="15" t="str">
+      <c r="A71" s="13">
+        <v>46317</v>
+      </c>
+      <c r="B71" s="14">
+        <v>480</v>
+      </c>
+      <c r="C71" s="14">
+        <v>60</v>
+      </c>
+      <c r="D71" s="14">
+        <v>150</v>
+      </c>
+      <c r="E71" s="14">
+        <v>200</v>
+      </c>
+      <c r="F71" s="14">
+        <v>200</v>
+      </c>
+      <c r="G71" s="14">
+        <v>4</v>
+      </c>
+      <c r="H71" s="14">
+        <v>350</v>
+      </c>
+      <c r="I71" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J71" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J71" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K71" s="16"/>
-      <c r="L71" s="16"/>
-      <c r="M71" s="16"/>
-      <c r="N71" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K71" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L71" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M71" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N71" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="13"/>

</xml_diff>

<commit_message>
update of 25th October
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BAC59F4-56A7-4A86-BCF3-1C57AC27661C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6542AA6-FDD9-4342-B2A3-98EEC035F3F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="120">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -389,6 +389,12 @@
   </si>
   <si>
     <t>good day</t>
+  </si>
+  <si>
+    <t>all ook</t>
+  </si>
+  <si>
+    <t>placement</t>
   </si>
 </sst>
 </file>
@@ -4212,70 +4218,142 @@
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A72" s="13"/>
-      <c r="B72" s="14"/>
-      <c r="C72" s="14"/>
-      <c r="D72" s="14"/>
-      <c r="E72" s="14"/>
-      <c r="F72" s="14"/>
-      <c r="G72" s="14"/>
-      <c r="H72" s="14"/>
-      <c r="I72" s="15" t="str">
+      <c r="A72" s="13">
+        <v>46318</v>
+      </c>
+      <c r="B72" s="14">
+        <v>480</v>
+      </c>
+      <c r="C72" s="14">
+        <v>60</v>
+      </c>
+      <c r="D72" s="14">
+        <v>150</v>
+      </c>
+      <c r="E72" s="14">
+        <v>200</v>
+      </c>
+      <c r="F72" s="14">
+        <v>250</v>
+      </c>
+      <c r="G72" s="14">
+        <v>5</v>
+      </c>
+      <c r="H72" s="14">
+        <v>300</v>
+      </c>
+      <c r="I72" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J72" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J72" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K72" s="16"/>
-      <c r="L72" s="16"/>
-      <c r="M72" s="16"/>
-      <c r="N72" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K72" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L72" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M72" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N72" s="17" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A73" s="13"/>
-      <c r="B73" s="14"/>
-      <c r="C73" s="14"/>
-      <c r="D73" s="14"/>
-      <c r="E73" s="14"/>
-      <c r="F73" s="14"/>
-      <c r="G73" s="14"/>
-      <c r="H73" s="14"/>
-      <c r="I73" s="15" t="str">
+      <c r="A73" s="13">
+        <v>46319</v>
+      </c>
+      <c r="B73" s="14">
+        <v>480</v>
+      </c>
+      <c r="C73" s="14">
+        <v>160</v>
+      </c>
+      <c r="D73" s="14">
+        <v>300</v>
+      </c>
+      <c r="E73" s="14">
+        <v>150</v>
+      </c>
+      <c r="F73" s="14">
+        <v>0</v>
+      </c>
+      <c r="G73" s="14">
+        <v>0</v>
+      </c>
+      <c r="H73" s="14">
+        <v>300</v>
+      </c>
+      <c r="I73" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J73" s="15" t="str">
+        <v>1390</v>
+      </c>
+      <c r="J73" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K73" s="16"/>
-      <c r="L73" s="16"/>
-      <c r="M73" s="16"/>
-      <c r="N73" s="17"/>
+        <v>50</v>
+      </c>
+      <c r="K73" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L73" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M73" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N73" s="17" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A74" s="13"/>
-      <c r="B74" s="14"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
-      <c r="G74" s="14"/>
-      <c r="H74" s="14"/>
-      <c r="I74" s="15" t="str">
+      <c r="A74" s="13">
+        <v>46320</v>
+      </c>
+      <c r="B74" s="14">
+        <v>480</v>
+      </c>
+      <c r="C74" s="14">
+        <v>160</v>
+      </c>
+      <c r="D74" s="14">
+        <v>300</v>
+      </c>
+      <c r="E74" s="14">
+        <v>150</v>
+      </c>
+      <c r="F74" s="14">
+        <v>0</v>
+      </c>
+      <c r="G74" s="14">
+        <v>0</v>
+      </c>
+      <c r="H74" s="14">
+        <v>300</v>
+      </c>
+      <c r="I74" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J74" s="15" t="str">
+        <v>1390</v>
+      </c>
+      <c r="J74" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K74" s="16"/>
-      <c r="L74" s="16"/>
-      <c r="M74" s="16"/>
-      <c r="N74" s="17"/>
+        <v>50</v>
+      </c>
+      <c r="K74" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L74" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M74" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N74" s="17" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" s="13"/>

</xml_diff>

<commit_message>
update og 28th October
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6542AA6-FDD9-4342-B2A3-98EEC035F3F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D062922-B48D-47F2-8E13-60326828DB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="123">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -395,6 +395,15 @@
   </si>
   <si>
     <t>placement</t>
+  </si>
+  <si>
+    <t>sick</t>
+  </si>
+  <si>
+    <t>doing something</t>
+  </si>
+  <si>
+    <t>just daily activities</t>
   </si>
 </sst>
 </file>
@@ -4356,70 +4365,142 @@
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A75" s="13"/>
-      <c r="B75" s="14"/>
-      <c r="C75" s="14"/>
-      <c r="D75" s="14"/>
-      <c r="E75" s="14"/>
-      <c r="F75" s="14"/>
-      <c r="G75" s="14"/>
-      <c r="H75" s="14"/>
-      <c r="I75" s="15" t="str">
+      <c r="A75" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B75" s="14">
+        <v>400</v>
+      </c>
+      <c r="C75" s="14">
+        <v>60</v>
+      </c>
+      <c r="D75" s="14">
+        <v>300</v>
+      </c>
+      <c r="E75" s="14">
+        <v>200</v>
+      </c>
+      <c r="F75" s="14">
+        <v>0</v>
+      </c>
+      <c r="G75" s="14">
+        <v>0</v>
+      </c>
+      <c r="H75" s="14">
+        <v>280</v>
+      </c>
+      <c r="I75" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J75" s="15" t="str">
+        <v>1240</v>
+      </c>
+      <c r="J75" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K75" s="16"/>
-      <c r="L75" s="16"/>
-      <c r="M75" s="16"/>
-      <c r="N75" s="17"/>
+        <v>200</v>
+      </c>
+      <c r="K75" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L75" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M75" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N75" s="17" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A76" s="13"/>
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="14"/>
-      <c r="F76" s="14"/>
-      <c r="G76" s="14"/>
-      <c r="H76" s="14"/>
-      <c r="I76" s="15" t="str">
+      <c r="A76" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B76" s="14">
+        <v>300</v>
+      </c>
+      <c r="C76" s="14">
+        <v>60</v>
+      </c>
+      <c r="D76" s="14">
+        <v>200</v>
+      </c>
+      <c r="E76" s="14">
+        <v>150</v>
+      </c>
+      <c r="F76" s="14">
+        <v>350</v>
+      </c>
+      <c r="G76" s="14">
+        <v>7</v>
+      </c>
+      <c r="H76" s="14">
+        <v>380</v>
+      </c>
+      <c r="I76" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J76" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J76" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K76" s="16"/>
-      <c r="L76" s="16"/>
-      <c r="M76" s="16"/>
-      <c r="N76" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K76" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L76" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M76" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N76" s="17" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A77" s="13"/>
-      <c r="B77" s="14"/>
-      <c r="C77" s="14"/>
-      <c r="D77" s="14"/>
-      <c r="E77" s="14"/>
-      <c r="F77" s="14"/>
-      <c r="G77" s="14"/>
-      <c r="H77" s="14"/>
-      <c r="I77" s="15" t="str">
+      <c r="A77" s="13">
+        <v>46323</v>
+      </c>
+      <c r="B77" s="14">
+        <v>400</v>
+      </c>
+      <c r="C77" s="14">
+        <v>60</v>
+      </c>
+      <c r="D77" s="14">
+        <v>200</v>
+      </c>
+      <c r="E77" s="14">
+        <v>150</v>
+      </c>
+      <c r="F77" s="14">
+        <v>350</v>
+      </c>
+      <c r="G77" s="14">
+        <v>7</v>
+      </c>
+      <c r="H77" s="14">
+        <v>280</v>
+      </c>
+      <c r="I77" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J77" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J77" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K77" s="16"/>
-      <c r="L77" s="16"/>
-      <c r="M77" s="16"/>
-      <c r="N77" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K77" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L77" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M77" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N77" s="17" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" s="13"/>

</xml_diff>

<commit_message>
update of 3oth October
</commit_message>
<xml_diff>
--- a/12600316.xlsx
+++ b/12600316.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piyus\OneDrive\Desktop\cap776\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D062922-B48D-47F2-8E13-60326828DB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D698CA-2DA3-446D-AF34-9012967EDCB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="124">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -404,6 +404,9 @@
   </si>
   <si>
     <t>just daily activities</t>
+  </si>
+  <si>
+    <t>working on CA project</t>
   </si>
 </sst>
 </file>
@@ -4503,48 +4506,96 @@
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A78" s="13"/>
-      <c r="B78" s="14"/>
-      <c r="C78" s="14"/>
-      <c r="D78" s="14"/>
-      <c r="E78" s="14"/>
-      <c r="F78" s="14"/>
-      <c r="G78" s="14"/>
-      <c r="H78" s="14"/>
-      <c r="I78" s="15" t="str">
+      <c r="A78" s="13">
+        <v>46324</v>
+      </c>
+      <c r="B78" s="14">
+        <v>480</v>
+      </c>
+      <c r="C78" s="14">
+        <v>100</v>
+      </c>
+      <c r="D78" s="14">
+        <v>190</v>
+      </c>
+      <c r="E78" s="14">
+        <v>270</v>
+      </c>
+      <c r="F78" s="14">
+        <v>200</v>
+      </c>
+      <c r="G78" s="14">
+        <v>4</v>
+      </c>
+      <c r="H78" s="14">
+        <v>200</v>
+      </c>
+      <c r="I78" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J78" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J78" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K78" s="16"/>
-      <c r="L78" s="16"/>
-      <c r="M78" s="16"/>
-      <c r="N78" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K78" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L78" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M78" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N78" s="17" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A79" s="13"/>
-      <c r="B79" s="14"/>
-      <c r="C79" s="14"/>
-      <c r="D79" s="14"/>
-      <c r="E79" s="14"/>
-      <c r="F79" s="14"/>
-      <c r="G79" s="14"/>
-      <c r="H79" s="14"/>
-      <c r="I79" s="15" t="str">
+      <c r="A79" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B79" s="14">
+        <v>480</v>
+      </c>
+      <c r="C79" s="14">
+        <v>100</v>
+      </c>
+      <c r="D79" s="14">
+        <v>180</v>
+      </c>
+      <c r="E79" s="14">
+        <v>310</v>
+      </c>
+      <c r="F79" s="14">
+        <v>250</v>
+      </c>
+      <c r="G79" s="14">
+        <v>5</v>
+      </c>
+      <c r="H79" s="14">
+        <v>120</v>
+      </c>
+      <c r="I79" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J79" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J79" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K79" s="16"/>
-      <c r="L79" s="16"/>
-      <c r="M79" s="16"/>
-      <c r="N79" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K79" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L79" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M79" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N79" s="17" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" s="13"/>

</xml_diff>